<commit_message>
add: test PlanillaReader match headers layout
</commit_message>
<xml_diff>
--- a/tests/FarmaLog.Ingesta.Tests/Fixtures/template-real.xlsx
+++ b/tests/FarmaLog.Ingesta.Tests/Fixtures/template-real.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\source\repos\FarmaLog\tests\FarmaLog.Ingesta.Tests\Fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF95B812-AB79-47B6-B87B-D0DB15A09093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD71AEBF-14D4-4361-8E67-E1FA08817716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{FCA89B08-6D76-4AEE-AECB-2AFEDABEE4FD}"/>
   </bookViews>
@@ -22,9 +22,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
-    <t>Número Pedido del Laboratorio</t>
-  </si>
-  <si>
     <t>Cuenta de Cliente</t>
   </si>
   <si>
@@ -41,9 +38,6 @@
 (opcional)</t>
   </si>
   <si>
-    <t>Código de Despacho</t>
-  </si>
-  <si>
     <t>Numero de Orden de Compra</t>
   </si>
   <si>
@@ -78,6 +72,12 @@
   </si>
   <si>
     <t>Pedido cargado por Ingesta</t>
+  </si>
+  <si>
+    <t>Numero Pedido del Laboratorio</t>
+  </si>
+  <si>
+    <t>Codigo de Despacho</t>
   </si>
 </sst>
 </file>
@@ -461,43 +461,43 @@
   <sheetData>
     <row r="1" spans="1:13" s="3" customFormat="1" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
@@ -515,26 +515,26 @@
         <v>10</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H2" s="1">
         <v>67539</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K2" s="6"/>
       <c r="L2" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">

</xml_diff>